<commit_message>
Refine BK RBI model: realistic franchise-heavy assumptions + auto-balancing base year
- Lower COGS to 30-32% of revenue (franchise/royalty-led mix) via new
  'COGS % of Revenue' assumption row; IS COGS now links to Assumptions
- Bring EBITDA margin to 30-32% (within the 20-35% QSR brief)
- Replace stale hard-coded opening-cash plug with an auto-computed base-year
  balancing figure so the balance sheet ties out for any assumptions
- Generator now writes the .xlsx into the repo directory (was sandbox root)

Balance sheet balances in all years; workbook validated (zip + XML + rels + cached formulas).

Co-authored-by: ilhom133 <198030582+ilhom133@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Burger_King_RBI_3_Statement_Model.xlsx
+++ b/Burger_King_RBI_3_Statement_Model.xlsx
@@ -173,19 +173,19 @@
         </is>
       </c>
       <c r="B5" s="4">
-        <v>0.35</v>
+        <v>0.3</v>
       </c>
       <c r="C5" s="4">
-        <v>0.355</v>
+        <v>0.305</v>
       </c>
       <c r="D5" s="4">
-        <v>0.36</v>
+        <v>0.31</v>
       </c>
       <c r="E5" s="4">
-        <v>0.365</v>
+        <v>0.315</v>
       </c>
       <c r="F5" s="4">
-        <v>0.37</v>
+        <v>0.32</v>
       </c>
     </row>
     <row r="6">
@@ -302,7 +302,28 @@
         <v>20696.589237</v>
       </c>
     </row>
-    <row r="11"/>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">COGS % of Revenue</t>
+        </is>
+      </c>
+      <c r="B11" s="4">
+        <v>0.32</v>
+      </c>
+      <c r="C11" s="4">
+        <v>0.315</v>
+      </c>
+      <c r="D11" s="4">
+        <v>0.31</v>
+      </c>
+      <c r="E11" s="4">
+        <v>0.305</v>
+      </c>
+      <c r="F11" s="4">
+        <v>0.3</v>
+      </c>
+    </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
@@ -327,7 +348,7 @@
     <row r="15">
       <c r="A15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">COGS = 40% of revenue; SG&amp;A is the plug so EBITDA = EBITDA Margin %.</t>
+          <t xml:space="preserve">COGS driven by COGS % of Revenue (row 11); SG&amp;A is the plug so EBITDA = EBITDA Margin %.</t>
         </is>
       </c>
     </row>
@@ -398,24 +419,24 @@
         </is>
       </c>
       <c r="B3" s="2">
-        <f>B2*0.4</f>
-        <v>800</v>
+        <f>B2*Assumptions!B11</f>
+        <v>640</v>
       </c>
       <c r="C3" s="2">
-        <f>C2*0.4</f>
-        <v>840</v>
+        <f>C2*Assumptions!C11</f>
+        <v>661.5</v>
       </c>
       <c r="D3" s="2">
-        <f>D2*0.4</f>
-        <v>877.8</v>
+        <f>D2*Assumptions!D11</f>
+        <v>680.295</v>
       </c>
       <c r="E3" s="2">
-        <f>E2*0.4</f>
-        <v>912.912</v>
+        <f>E2*Assumptions!E11</f>
+        <v>696.0954</v>
       </c>
       <c r="F3" s="2">
-        <f>F2*0.4</f>
-        <v>949.42848</v>
+        <f>F2*Assumptions!F11</f>
+        <v>712.07136</v>
       </c>
     </row>
     <row r="4">
@@ -426,23 +447,23 @@
       </c>
       <c r="B4" s="2">
         <f>B2-B3</f>
-        <v>1200</v>
+        <v>1360</v>
       </c>
       <c r="C4" s="2">
         <f>C2-C3</f>
-        <v>1260</v>
+        <v>1438.5</v>
       </c>
       <c r="D4" s="2">
         <f>D2-D3</f>
-        <v>1316.7</v>
+        <v>1514.205</v>
       </c>
       <c r="E4" s="2">
         <f>E2-E3</f>
-        <v>1369.368</v>
+        <v>1586.1846</v>
       </c>
       <c r="F4" s="2">
         <f>F2-F3</f>
-        <v>1424.14272</v>
+        <v>1661.49984</v>
       </c>
     </row>
     <row r="5">
@@ -453,23 +474,23 @@
       </c>
       <c r="B5" s="4">
         <f>B4/B2</f>
-        <v>0.6</v>
+        <v>0.68</v>
       </c>
       <c r="C5" s="4">
         <f>C4/C2</f>
-        <v>0.6</v>
+        <v>0.685</v>
       </c>
       <c r="D5" s="4">
         <f>D4/D2</f>
-        <v>0.6</v>
+        <v>0.69</v>
       </c>
       <c r="E5" s="4">
         <f>E4/E2</f>
-        <v>0.6</v>
+        <v>0.695</v>
       </c>
       <c r="F5" s="4">
         <f>F4/F2</f>
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="6">
@@ -480,23 +501,23 @@
       </c>
       <c r="B6" s="2">
         <f>B4-B7</f>
-        <v>500</v>
+        <v>760</v>
       </c>
       <c r="C6" s="2">
         <f>C4-C7</f>
-        <v>514.5</v>
+        <v>798</v>
       </c>
       <c r="D6" s="2">
         <f>D4-D7</f>
-        <v>526.68</v>
+        <v>833.91</v>
       </c>
       <c r="E6" s="2">
         <f>E4-E7</f>
-        <v>536.3358</v>
+        <v>867.2664</v>
       </c>
       <c r="F6" s="2">
         <f>F4-F7</f>
-        <v>545.921376</v>
+        <v>901.957056</v>
       </c>
     </row>
     <row r="7">
@@ -507,23 +528,23 @@
       </c>
       <c r="B7" s="3">
         <f>B2*Assumptions!B5</f>
-        <v>700</v>
+        <v>600</v>
       </c>
       <c r="C7" s="3">
         <f>C2*Assumptions!C5</f>
-        <v>745.5</v>
+        <v>640.5</v>
       </c>
       <c r="D7" s="3">
         <f>D2*Assumptions!D5</f>
-        <v>790.02</v>
+        <v>680.295</v>
       </c>
       <c r="E7" s="3">
         <f>E2*Assumptions!E5</f>
-        <v>833.0322</v>
+        <v>718.9182</v>
       </c>
       <c r="F7" s="3">
         <f>F2*Assumptions!F5</f>
-        <v>878.221344</v>
+        <v>759.542784</v>
       </c>
     </row>
     <row r="8">
@@ -561,23 +582,23 @@
       </c>
       <c r="B9" s="3">
         <f>B7-B8</f>
-        <v>600</v>
+        <v>500</v>
       </c>
       <c r="C9" s="3">
         <f>C7-C8</f>
-        <v>640.5</v>
+        <v>535.5</v>
       </c>
       <c r="D9" s="3">
         <f>D7-D8</f>
-        <v>680.295</v>
+        <v>570.57</v>
       </c>
       <c r="E9" s="3">
         <f>E7-E8</f>
-        <v>718.9182</v>
+        <v>604.8042</v>
       </c>
       <c r="F9" s="3">
         <f>F7-F8</f>
-        <v>759.542784</v>
+        <v>640.864224</v>
       </c>
     </row>
     <row r="10">
@@ -615,23 +636,23 @@
       </c>
       <c r="B11" s="2">
         <f>B9-B10</f>
-        <v>425</v>
+        <v>325</v>
       </c>
       <c r="C11" s="2">
         <f>C9-C10</f>
-        <v>470.5</v>
+        <v>365.5</v>
       </c>
       <c r="D11" s="2">
         <f>D9-D10</f>
-        <v>515.295</v>
+        <v>405.57</v>
       </c>
       <c r="E11" s="2">
         <f>E9-E10</f>
-        <v>558.9182</v>
+        <v>444.8042</v>
       </c>
       <c r="F11" s="2">
         <f>F9-F10</f>
-        <v>604.542784</v>
+        <v>485.864224</v>
       </c>
     </row>
     <row r="12">
@@ -642,23 +663,23 @@
       </c>
       <c r="B12" s="2">
         <f>B11*Assumptions!B7</f>
-        <v>89.25</v>
+        <v>68.25</v>
       </c>
       <c r="C12" s="2">
         <f>C11*Assumptions!C7</f>
-        <v>98.805</v>
+        <v>76.755</v>
       </c>
       <c r="D12" s="2">
         <f>D11*Assumptions!D7</f>
-        <v>108.21195</v>
+        <v>85.1697</v>
       </c>
       <c r="E12" s="2">
         <f>E11*Assumptions!E7</f>
-        <v>117.372822</v>
+        <v>93.408882</v>
       </c>
       <c r="F12" s="2">
         <f>F11*Assumptions!F7</f>
-        <v>126.953985</v>
+        <v>102.031487</v>
       </c>
     </row>
     <row r="13">
@@ -669,23 +690,23 @@
       </c>
       <c r="B13" s="3">
         <f>B11-B12</f>
-        <v>335.75</v>
+        <v>256.75</v>
       </c>
       <c r="C13" s="3">
         <f>C11-C12</f>
-        <v>371.695</v>
+        <v>288.745</v>
       </c>
       <c r="D13" s="3">
         <f>D11-D12</f>
-        <v>407.08305</v>
+        <v>320.4003</v>
       </c>
       <c r="E13" s="3">
         <f>E11-E12</f>
-        <v>441.545378</v>
+        <v>351.395318</v>
       </c>
       <c r="F13" s="3">
         <f>F11-F12</f>
-        <v>477.588799</v>
+        <v>383.832737</v>
       </c>
     </row>
   </sheetData>
@@ -741,19 +762,19 @@
       </c>
       <c r="C3" s="2">
         <f>CF!C13</f>
-        <v>941.9265</v>
+        <v>900.4515</v>
       </c>
       <c r="D3" s="2">
         <f>CF!D13</f>
-        <v>1050.490333</v>
+        <v>965.673957</v>
       </c>
       <c r="E3" s="2">
         <f>CF!E13</f>
-        <v>1174.700143</v>
+        <v>1044.808738</v>
       </c>
       <c r="F3" s="2">
         <f>CF!F13</f>
-        <v>1315.784533</v>
+        <v>1139.015097</v>
       </c>
     </row>
     <row r="4">
@@ -846,19 +867,19 @@
       </c>
       <c r="C7" s="3">
         <f>SUM(C3:C6)</f>
-        <v>1088.9265</v>
+        <v>1047.4515</v>
       </c>
       <c r="D7" s="3">
         <f>SUM(D3:D6)</f>
-        <v>1204.105333</v>
+        <v>1119.288957</v>
       </c>
       <c r="E7" s="3">
         <f>SUM(E3:E6)</f>
-        <v>1334.459743</v>
+        <v>1204.568338</v>
       </c>
       <c r="F7" s="3">
         <f>SUM(F3:F6)</f>
-        <v>1481.934517</v>
+        <v>1305.165081</v>
       </c>
     </row>
     <row r="8">
@@ -1004,19 +1025,19 @@
       </c>
       <c r="C13" s="3">
         <f>C7+C12</f>
-        <v>9986.8475</v>
+        <v>9945.3725</v>
       </c>
       <c r="D13" s="3">
         <f>D7+D12</f>
-        <v>10100.784025</v>
+        <v>10015.96765</v>
       </c>
       <c r="E13" s="3">
         <f>E7+E12</f>
-        <v>10231.212514</v>
+        <v>10101.321109</v>
       </c>
       <c r="F13" s="3">
         <f>F7+F12</f>
-        <v>10380.048946</v>
+        <v>10203.279509</v>
       </c>
     </row>
     <row r="14">
@@ -1333,19 +1354,19 @@
       </c>
       <c r="C27" s="2">
         <f>B27+IS!C13+CF!C9</f>
-        <v>3155.8475</v>
+        <v>3114.3725</v>
       </c>
       <c r="D27" s="2">
         <f>C27+IS!D13+CF!D9</f>
-        <v>3359.389025</v>
+        <v>3274.57265</v>
       </c>
       <c r="E27" s="2">
         <f>D27+IS!E13+CF!E9</f>
-        <v>3580.161714</v>
+        <v>3450.270309</v>
       </c>
       <c r="F27" s="2">
         <f>E27+IS!F13+CF!F9</f>
-        <v>3818.956114</v>
+        <v>3642.186677</v>
       </c>
     </row>
     <row r="28">
@@ -1412,19 +1433,19 @@
       </c>
       <c r="C30" s="3">
         <f>C26+C27+C28+C29</f>
-        <v>4755.8475</v>
+        <v>4714.3725</v>
       </c>
       <c r="D30" s="3">
         <f>D26+D27+D28+D29</f>
-        <v>4959.389025</v>
+        <v>4874.57265</v>
       </c>
       <c r="E30" s="3">
         <f>E26+E27+E28+E29</f>
-        <v>5180.161714</v>
+        <v>5050.270309</v>
       </c>
       <c r="F30" s="3">
         <f>F26+F27+F28+F29</f>
-        <v>5418.956114</v>
+        <v>5242.186677</v>
       </c>
     </row>
     <row r="31">
@@ -1439,19 +1460,19 @@
       </c>
       <c r="C31" s="3">
         <f>C24+C30</f>
-        <v>9986.8475</v>
+        <v>9945.3725</v>
       </c>
       <c r="D31" s="3">
         <f>D24+D30</f>
-        <v>10100.784025</v>
+        <v>10015.96765</v>
       </c>
       <c r="E31" s="3">
         <f>E24+E30</f>
-        <v>10231.212514</v>
+        <v>10101.321109</v>
       </c>
       <c r="F31" s="3">
         <f>F24+F30</f>
-        <v>10380.048946</v>
+        <v>10203.279509</v>
       </c>
     </row>
     <row r="32">
@@ -1523,23 +1544,23 @@
       </c>
       <c r="B2" s="2">
         <f>IS!B13</f>
-        <v>335.75</v>
+        <v>256.75</v>
       </c>
       <c r="C2" s="2">
         <f>IS!C13</f>
-        <v>371.695</v>
+        <v>288.745</v>
       </c>
       <c r="D2" s="2">
         <f>IS!D13</f>
-        <v>407.08305</v>
+        <v>320.4003</v>
       </c>
       <c r="E2" s="2">
         <f>IS!E13</f>
-        <v>441.545378</v>
+        <v>351.395318</v>
       </c>
       <c r="F2" s="2">
         <f>IS!F13</f>
-        <v>477.588799</v>
+        <v>383.832737</v>
       </c>
     </row>
     <row r="3">
@@ -1603,23 +1624,23 @@
       </c>
       <c r="B5" s="3">
         <f>B2+B3+B4</f>
-        <v>439.56</v>
+        <v>360.56</v>
       </c>
       <c r="C5" s="3">
         <f>C2+C3+C4</f>
-        <v>480.695</v>
+        <v>397.745</v>
       </c>
       <c r="D5" s="3">
         <f>D2+D3+D4</f>
-        <v>520.58805</v>
+        <v>433.9053</v>
       </c>
       <c r="E5" s="3">
         <f>E2+E3+E4</f>
-        <v>559.170578</v>
+        <v>469.020518</v>
       </c>
       <c r="F5" s="3">
         <f>F2+F3+F4</f>
-        <v>599.919007</v>
+        <v>506.162945</v>
       </c>
     </row>
     <row r="6">
@@ -1710,23 +1731,23 @@
       </c>
       <c r="B9" s="2">
         <f>-0.5*IS!B13</f>
-        <v>-167.875</v>
+        <v>-128.375</v>
       </c>
       <c r="C9" s="2">
         <f>-0.5*IS!C13</f>
-        <v>-185.8475</v>
+        <v>-144.3725</v>
       </c>
       <c r="D9" s="2">
         <f>-0.5*IS!D13</f>
-        <v>-203.541525</v>
+        <v>-160.20015</v>
       </c>
       <c r="E9" s="2">
         <f>-0.5*IS!E13</f>
-        <v>-220.772689</v>
+        <v>-175.697659</v>
       </c>
       <c r="F9" s="2">
         <f>-0.5*IS!F13</f>
-        <v>-238.7944</v>
+        <v>-191.916368</v>
       </c>
     </row>
     <row r="10">
@@ -1737,23 +1758,23 @@
       </c>
       <c r="B10" s="3">
         <f>B8+B9</f>
-        <v>-267.875</v>
+        <v>-228.375</v>
       </c>
       <c r="C10" s="3">
         <f>C8+C9</f>
-        <v>-285.8475</v>
+        <v>-244.3725</v>
       </c>
       <c r="D10" s="3">
         <f>D8+D9</f>
-        <v>-303.541525</v>
+        <v>-260.20015</v>
       </c>
       <c r="E10" s="3">
         <f>E8+E9</f>
-        <v>-320.772689</v>
+        <v>-275.697659</v>
       </c>
       <c r="F10" s="3">
         <f>F8+F9</f>
-        <v>-338.7944</v>
+        <v>-291.916368</v>
       </c>
     </row>
     <row r="11">
@@ -1764,23 +1785,23 @@
       </c>
       <c r="B11" s="3">
         <f>B5+B7+B10</f>
-        <v>74.185</v>
+        <v>34.685</v>
       </c>
       <c r="C11" s="3">
         <f>C5+C7+C10</f>
-        <v>91.9265</v>
+        <v>50.4515</v>
       </c>
       <c r="D11" s="3">
         <f>D5+D7+D10</f>
-        <v>108.563832</v>
+        <v>65.222457</v>
       </c>
       <c r="E11" s="3">
         <f>E5+E7+E10</f>
-        <v>124.20981</v>
+        <v>79.13478</v>
       </c>
       <c r="F11" s="3">
         <f>F5+F7+F10</f>
-        <v>141.08439</v>
+        <v>94.206359</v>
       </c>
     </row>
     <row r="12">
@@ -1790,7 +1811,7 @@
         </is>
       </c>
       <c r="B12" s="2">
-        <v>775.815</v>
+        <v>815.315</v>
       </c>
       <c r="C12" s="2">
         <f>B13</f>
@@ -1798,15 +1819,15 @@
       </c>
       <c r="D12" s="2">
         <f>C13</f>
-        <v>941.9265</v>
+        <v>900.4515</v>
       </c>
       <c r="E12" s="2">
         <f>D13</f>
-        <v>1050.490333</v>
+        <v>965.673957</v>
       </c>
       <c r="F12" s="2">
         <f>E13</f>
-        <v>1174.700143</v>
+        <v>1044.808738</v>
       </c>
     </row>
     <row r="13">
@@ -1821,19 +1842,19 @@
       </c>
       <c r="C13" s="3">
         <f>C12+C11</f>
-        <v>941.9265</v>
+        <v>900.4515</v>
       </c>
       <c r="D13" s="3">
         <f>D12+D11</f>
-        <v>1050.490333</v>
+        <v>965.673957</v>
       </c>
       <c r="E13" s="3">
         <f>E12+E11</f>
-        <v>1174.700143</v>
+        <v>1044.808738</v>
       </c>
       <c r="F13" s="3">
         <f>F12+F11</f>
-        <v>1315.784533</v>
+        <v>1139.015097</v>
       </c>
     </row>
     <row r="14">
@@ -1928,23 +1949,23 @@
       </c>
       <c r="B3" s="4">
         <f>IS!B7/IS!B2</f>
-        <v>0.35</v>
+        <v>0.3</v>
       </c>
       <c r="C3" s="4">
         <f>IS!C7/IS!C2</f>
-        <v>0.355</v>
+        <v>0.305</v>
       </c>
       <c r="D3" s="4">
         <f>IS!D7/IS!D2</f>
-        <v>0.36</v>
+        <v>0.31</v>
       </c>
       <c r="E3" s="4">
         <f>IS!E7/IS!E2</f>
-        <v>0.365</v>
+        <v>0.315</v>
       </c>
       <c r="F3" s="4">
         <f>IS!F7/IS!F2</f>
-        <v>0.37</v>
+        <v>0.32</v>
       </c>
     </row>
     <row r="4">
@@ -1955,23 +1976,23 @@
       </c>
       <c r="B4" s="4">
         <f>IS!B13/IS!B2</f>
-        <v>0.167875</v>
+        <v>0.128375</v>
       </c>
       <c r="C4" s="4">
         <f>IS!C13/IS!C2</f>
-        <v>0.176998</v>
+        <v>0.137498</v>
       </c>
       <c r="D4" s="4">
         <f>IS!D13/IS!D2</f>
-        <v>0.185502</v>
+        <v>0.146002</v>
       </c>
       <c r="E4" s="4">
         <f>IS!E13/IS!E2</f>
-        <v>0.193467</v>
+        <v>0.153967</v>
       </c>
       <c r="F4" s="4">
         <f>IS!F13/IS!F2</f>
-        <v>0.201211</v>
+        <v>0.161711</v>
       </c>
     </row>
     <row r="5">
@@ -1982,23 +2003,23 @@
       </c>
       <c r="B5" s="7">
         <f>(BS!B17+BS!B20)/IS!B7</f>
-        <v>5</v>
+        <v>5.833333</v>
       </c>
       <c r="C5" s="7">
         <f>(BS!C17+BS!C20)/IS!C7</f>
-        <v>4.560698</v>
+        <v>5.308353</v>
       </c>
       <c r="D5" s="7">
         <f>(BS!D17+BS!D20)/IS!D7</f>
-        <v>4.177109</v>
+        <v>4.850837</v>
       </c>
       <c r="E5" s="7">
         <f>(BS!E17+BS!E20)/IS!E7</f>
-        <v>3.841388</v>
+        <v>4.451132</v>
       </c>
       <c r="F5" s="7">
         <f>(BS!F17+BS!F20)/IS!F7</f>
-        <v>3.529862</v>
+        <v>4.081403</v>
       </c>
     </row>
     <row r="6">
@@ -2009,23 +2030,23 @@
       </c>
       <c r="B6" s="7">
         <f>IS!B9/IS!B10</f>
-        <v>3.428571</v>
+        <v>2.857143</v>
       </c>
       <c r="C6" s="7">
         <f>IS!C9/IS!C10</f>
-        <v>3.767647</v>
+        <v>3.15</v>
       </c>
       <c r="D6" s="7">
         <f>IS!D9/IS!D10</f>
-        <v>4.123</v>
+        <v>3.458</v>
       </c>
       <c r="E6" s="7">
         <f>IS!E9/IS!E10</f>
-        <v>4.493239</v>
+        <v>3.780026</v>
       </c>
       <c r="F6" s="7">
         <f>IS!F9/IS!F10</f>
-        <v>4.900276</v>
+        <v>4.134608</v>
       </c>
     </row>
     <row r="7">
@@ -2036,23 +2057,23 @@
       </c>
       <c r="B7" s="4">
         <f>IS!B13/BS!B30</f>
-        <v>0.073468</v>
+        <v>0.056182</v>
       </c>
       <c r="C7" s="4">
         <f>IS!C13/BS!C30</f>
-        <v>0.078155</v>
+        <v>0.061248</v>
       </c>
       <c r="D7" s="4">
         <f>IS!D13/BS!D30</f>
-        <v>0.082083</v>
+        <v>0.065729</v>
       </c>
       <c r="E7" s="4">
         <f>IS!E13/BS!E30</f>
-        <v>0.085238</v>
+        <v>0.06958</v>
       </c>
       <c r="F7" s="4">
         <f>IS!F13/BS!F30</f>
-        <v>0.088133</v>
+        <v>0.07322</v>
       </c>
     </row>
     <row r="8">
@@ -2063,23 +2084,23 @@
       </c>
       <c r="B8" s="3">
         <f>CF!B5+CF!B6</f>
-        <v>342.06</v>
+        <v>263.06</v>
       </c>
       <c r="C8" s="3">
         <f>CF!C5+CF!C6</f>
-        <v>377.774</v>
+        <v>294.824</v>
       </c>
       <c r="D8" s="3">
         <f>CF!D5+CF!D6</f>
-        <v>412.105357</v>
+        <v>325.422607</v>
       </c>
       <c r="E8" s="3">
         <f>CF!E5+CF!E6</f>
-        <v>444.982499</v>
+        <v>354.832439</v>
       </c>
       <c r="F8" s="3">
         <f>CF!F5+CF!F6</f>
-        <v>479.87879</v>
+        <v>386.122727</v>
       </c>
     </row>
   </sheetData>

</xml_diff>